<commit_message>
Manuscript: drop the SRS/SCQ supplementary figure, add Supplementary Table 10 (slopes by autism status)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Supplementary_Tables.xlsx
+++ b/Supplementary_Tables.xlsx
@@ -16,13 +16,14 @@
     <sheet name="Supplementary Table 8" sheetId="27" r:id="rId8"/>
     <sheet name="Supplementary Table 9" sheetId="29" state="visible" r:id="rId10"/>
     <sheet name="Supplementary Table 9 prev" sheetId="30" state="visible" r:id="rId11"/>
+    <sheet name="Supplementary Table 10" sheetId="31" state="visible" r:id="rId12"/>
     <sheet name="notes" sheetId="28" state="visible" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3235" uniqueCount="3235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3247" uniqueCount="3247">
   <si>
     <t xml:space="preserve">Trait</t>
   </si>
@@ -9727,6 +9728,42 @@
   </si>
   <si>
     <t xml:space="preserve">weight_loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">variant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diff_se</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diff_p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ci_lo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ci_hi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSC siblings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSC parents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unaffected relatives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">all carriers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">non-ASD carriers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASD-adjusted</t>
   </si>
 </sst>
 </file>
@@ -18072,6 +18109,2425 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3235</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3216</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3201</v>
+      </c>
+      <c r="G1" t="s">
+        <v>392</v>
+      </c>
+      <c r="H1" t="s">
+        <v>3236</v>
+      </c>
+      <c r="I1" t="s">
+        <v>3237</v>
+      </c>
+      <c r="J1" t="s">
+        <v>3238</v>
+      </c>
+      <c r="K1" t="s">
+        <v>3239</v>
+      </c>
+      <c r="L1" t="s">
+        <v>3240</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3241</v>
+      </c>
+      <c r="C2" t="s">
+        <v>366</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1578</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.00359107989029812</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.0197565891267438</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.855789645176673</v>
+      </c>
+      <c r="H2"/>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2" t="n">
+        <v>-0.0351318347981198</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0423139945787161</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>197</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3242</v>
+      </c>
+      <c r="C3" t="s">
+        <v>366</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3891</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0219380711802651</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0160263988408617</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.171118754208664</v>
+      </c>
+      <c r="H3"/>
+      <c r="I3"/>
+      <c r="J3"/>
+      <c r="K3" t="n">
+        <v>-0.00947367054782372</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.053349812908354</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3243</v>
+      </c>
+      <c r="C4" t="s">
+        <v>366</v>
+      </c>
+      <c r="D4" t="n">
+        <v>5469</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0144646962977217</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0124565070982652</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.245604782095427</v>
+      </c>
+      <c r="H4"/>
+      <c r="I4"/>
+      <c r="J4"/>
+      <c r="K4" t="n">
+        <v>-0.00995005761487815</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.0388794502103216</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>366</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2065</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0252732831747767</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.0306879724667344</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.410286820964376</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.0266919665351804</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.0332298520192682</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.421854108387597</v>
+      </c>
+      <c r="K5" t="n">
+        <v>-0.0348751428600228</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.0854217092095761</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>197</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D6" t="n">
+        <v>79</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.17601213225003</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.20225292606236</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.386900142322132</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.168314230044467</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.084592215195568</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.0466717175229145</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-0.220403602832196</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.572427867332256</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D7" t="n">
+        <v>43</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.192621095031013</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.185391223741184</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.305045710583397</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-0.208917576356822</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.103737411581686</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.0440678341496846</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-0.555987893563733</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.170745703501707</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D8" t="n">
+        <v>76</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.0880580925256814</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.153478586404725</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.567926048615496</v>
+      </c>
+      <c r="H8"/>
+      <c r="I8"/>
+      <c r="J8"/>
+      <c r="K8" t="n">
+        <v>-0.21275993682758</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.388876121878943</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>197</v>
+      </c>
+      <c r="B9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D9" t="n">
+        <v>34</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.53410511697608</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.253409835391944</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.0434547027782688</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.508332343284307</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.12182354643802</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.0000305670495853483</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.0374218396078695</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1.03078839434429</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>197</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D10" t="n">
+        <v>18</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.049000669085545</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.242659157569216</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.842941188657831</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.010682306446026</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.161873340585102</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.947386797402947</v>
+      </c>
+      <c r="K10" t="n">
+        <v>-0.426611279750119</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.524612617921209</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>197</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D11" t="n">
+        <v>33</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.451053530028226</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.205903786467028</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.0369976449721818</v>
+      </c>
+      <c r="H11"/>
+      <c r="I11"/>
+      <c r="J11"/>
+      <c r="K11" t="n">
+        <v>0.0474821085528508</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.854624951503602</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>197</v>
+      </c>
+      <c r="B12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D12" t="n">
+        <v>207</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.257871731484011</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.098832538938323</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.00975503136949215</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.238801691021674</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.0521266424848927</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.00000472274601642412</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.0641599551648983</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.451583507803124</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>197</v>
+      </c>
+      <c r="B13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D13" t="n">
+        <v>150</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.215480232301596</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.103894225860759</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.039843539354302</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.208658828980928</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.0607697546196685</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.000599946018881335</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.0118475496145086</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.419112914988683</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>197</v>
+      </c>
+      <c r="B14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D14" t="n">
+        <v>193</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.141105204358805</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.0934475155095042</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.132729574474166</v>
+      </c>
+      <c r="H14"/>
+      <c r="I14"/>
+      <c r="J14"/>
+      <c r="K14" t="n">
+        <v>-0.0420519260398234</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.324262334757433</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>197</v>
+      </c>
+      <c r="B15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D15" t="n">
+        <v>66</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.0806483173564682</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.235390472963164</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.73302859542266</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-0.0599872792534352</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.107601112234906</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.577210638928828</v>
+      </c>
+      <c r="K15" t="n">
+        <v>-0.380717009651333</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.542013644364269</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>197</v>
+      </c>
+      <c r="B16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D16" t="n">
+        <v>49</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.0167671277397135</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.2245526835259</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.940801840993148</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-0.000348028106837701</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.117705793711287</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.997640955250475</v>
+      </c>
+      <c r="K16" t="n">
+        <v>-0.423356131971051</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.456890387450478</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>197</v>
+      </c>
+      <c r="B17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D17" t="n">
+        <v>63</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-0.0729121942350559</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.191597879913793</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.704905361668141</v>
+      </c>
+      <c r="H17"/>
+      <c r="I17"/>
+      <c r="J17"/>
+      <c r="K17" t="n">
+        <v>-0.44844403886609</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.302619650395978</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>197</v>
+      </c>
+      <c r="B18" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D18" t="n">
+        <v>386</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.239445792419842</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.0807499299372799</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.00321602392590051</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.216173341395559</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.044464770985633</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.00000119445958108421</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.0811759297427737</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.397715655096911</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>197</v>
+      </c>
+      <c r="B19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C19" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D19" t="n">
+        <v>260</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.109050557396361</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.0815549207541092</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.182379448812867</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.0959027394816015</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.0491455399086562</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.0510579928467547</v>
+      </c>
+      <c r="K19" t="n">
+        <v>-0.0507970872816926</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.268898202074415</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>197</v>
+      </c>
+      <c r="B20" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D20" t="n">
+        <v>365</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.137022981238078</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.0703401256137758</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.052198409582294</v>
+      </c>
+      <c r="H20"/>
+      <c r="I20"/>
+      <c r="J20"/>
+      <c r="K20" t="n">
+        <v>-0.000843664964922469</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.274889627441079</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>271</v>
+      </c>
+      <c r="B21" t="s">
+        <v>3241</v>
+      </c>
+      <c r="C21" t="s">
+        <v>366</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1134</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.00856914679227391</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.0226852161862663</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.705693577169033</v>
+      </c>
+      <c r="H21"/>
+      <c r="I21"/>
+      <c r="J21"/>
+      <c r="K21" t="n">
+        <v>-0.0358938769328081</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.0530321705173559</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>271</v>
+      </c>
+      <c r="B22" t="s">
+        <v>3243</v>
+      </c>
+      <c r="C22" t="s">
+        <v>366</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1134</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.00856914679227391</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.0226852161862663</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.705693577169033</v>
+      </c>
+      <c r="H22"/>
+      <c r="I22"/>
+      <c r="J22"/>
+      <c r="K22" t="n">
+        <v>-0.0358938769328081</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.0530321705173559</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>271</v>
+      </c>
+      <c r="B23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" t="s">
+        <v>366</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1503</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.0257046739413946</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.0666817294225028</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.699934333804886</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.0214026827920657</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.0820607042684143</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.794255428864621</v>
+      </c>
+      <c r="K23" t="n">
+        <v>-0.104991515726711</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.1564008636095</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>271</v>
+      </c>
+      <c r="B24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D24" t="n">
+        <v>60</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.440485814903169</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.314170744204802</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.166320276551054</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.260934851498014</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.123031356921777</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.0341398485406325</v>
+      </c>
+      <c r="K24" t="n">
+        <v>-0.175288843738242</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1.05626047354458</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>271</v>
+      </c>
+      <c r="B25" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D25" t="n">
+        <v>30</v>
+      </c>
+      <c r="E25" t="n">
+        <v>-0.0197565492508892</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.430541591394667</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.96374711826497</v>
+      </c>
+      <c r="H25" t="n">
+        <v>-0.110860730456006</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.163186496683628</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.49705229599999</v>
+      </c>
+      <c r="K25" t="n">
+        <v>-0.863618068384436</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.824104969882658</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>271</v>
+      </c>
+      <c r="B26" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D26" t="n">
+        <v>58</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.409006916290119</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.247704095036809</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.104534918534814</v>
+      </c>
+      <c r="H26"/>
+      <c r="I26"/>
+      <c r="J26"/>
+      <c r="K26" t="n">
+        <v>-0.0764931099820263</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0.894506942562265</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>271</v>
+      </c>
+      <c r="B27" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D27" t="n">
+        <v>21</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.332185960302529</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.497696655210681</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.512953825503438</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.477249584335799</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.165127675861294</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.00392297795159589</v>
+      </c>
+      <c r="K27" t="n">
+        <v>-0.643299483910407</v>
+      </c>
+      <c r="L27" t="n">
+        <v>1.30767140451546</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>271</v>
+      </c>
+      <c r="B28" t="s">
+        <v>40</v>
+      </c>
+      <c r="C28" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D28" t="n">
+        <v>21</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.338113573185118</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.473483626274689</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.484856963446141</v>
+      </c>
+      <c r="H28"/>
+      <c r="I28"/>
+      <c r="J28"/>
+      <c r="K28" t="n">
+        <v>-0.589914334313272</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1.26614148068351</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>271</v>
+      </c>
+      <c r="B29" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D29" t="n">
+        <v>169</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.288361481123169</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.152075870937024</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.0596878926104265</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.27440160821743</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.0833957208182628</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.00102764857100989</v>
+      </c>
+      <c r="K29" t="n">
+        <v>-0.00970722591339851</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0.586430188159736</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>271</v>
+      </c>
+      <c r="B30" t="s">
+        <v>54</v>
+      </c>
+      <c r="C30" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D30" t="n">
+        <v>118</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.0645602056386988</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.141163992075907</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.648299190736309</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.0472740940478454</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.0821570192777715</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.565117482504991</v>
+      </c>
+      <c r="K30" t="n">
+        <v>-0.212121218830079</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0.341241630107477</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>271</v>
+      </c>
+      <c r="B31" t="s">
+        <v>54</v>
+      </c>
+      <c r="C31" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D31" t="n">
+        <v>156</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.160400435356832</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.135558343597944</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.238575037898914</v>
+      </c>
+      <c r="H31"/>
+      <c r="I31"/>
+      <c r="J31"/>
+      <c r="K31" t="n">
+        <v>-0.105293918095138</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0.426094788808803</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>271</v>
+      </c>
+      <c r="B32" t="s">
+        <v>67</v>
+      </c>
+      <c r="C32" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D32" t="n">
+        <v>50</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.449680266300944</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.370594189892096</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.231038559235251</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.379643224015863</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.128860457662685</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.00328102086074221</v>
+      </c>
+      <c r="K32" t="n">
+        <v>-0.276684345887564</v>
+      </c>
+      <c r="L32" t="n">
+        <v>1.17604487848945</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>271</v>
+      </c>
+      <c r="B33" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D33" t="n">
+        <v>40</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.534919794617647</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.384910859584139</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.172918745206875</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.459829235897054</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.132779502276848</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.000553359612664009</v>
+      </c>
+      <c r="K33" t="n">
+        <v>-0.219505490167266</v>
+      </c>
+      <c r="L33" t="n">
+        <v>1.28934507940256</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>271</v>
+      </c>
+      <c r="B34" t="s">
+        <v>67</v>
+      </c>
+      <c r="C34" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D34" t="n">
+        <v>47</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.429911197742887</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.352102324704975</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.228745037374161</v>
+      </c>
+      <c r="H34"/>
+      <c r="I34"/>
+      <c r="J34"/>
+      <c r="K34" t="n">
+        <v>-0.260209358678865</v>
+      </c>
+      <c r="L34" t="n">
+        <v>1.12003175416464</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>271</v>
+      </c>
+      <c r="B35" t="s">
+        <v>103</v>
+      </c>
+      <c r="C35" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D35" t="n">
+        <v>300</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.334425620888574</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.127412593523474</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.00912635765987333</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.337346509144931</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.082903439750026</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.0000497833222378138</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.0846969375825653</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0.584154304194582</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>271</v>
+      </c>
+      <c r="B36" t="s">
+        <v>103</v>
+      </c>
+      <c r="C36" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D36" t="n">
+        <v>199</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.155138765956143</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.131143613426311</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.238288440461884</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.158772531439226</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.0791172738657242</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.0449748959506755</v>
+      </c>
+      <c r="K36" t="n">
+        <v>-0.101902716359427</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0.412180248271713</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>271</v>
+      </c>
+      <c r="B37" t="s">
+        <v>103</v>
+      </c>
+      <c r="C37" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D37" t="n">
+        <v>282</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.267469375065971</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.112523789654808</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.0181420750480226</v>
+      </c>
+      <c r="H37"/>
+      <c r="I37"/>
+      <c r="J37"/>
+      <c r="K37" t="n">
+        <v>0.0469227473425486</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0.488016002789394</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>340</v>
+      </c>
+      <c r="B38" t="s">
+        <v>3241</v>
+      </c>
+      <c r="C38" t="s">
+        <v>366</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38"/>
+      <c r="F38"/>
+      <c r="G38"/>
+      <c r="H38"/>
+      <c r="I38"/>
+      <c r="J38"/>
+      <c r="K38"/>
+      <c r="L38"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>340</v>
+      </c>
+      <c r="B39" t="s">
+        <v>3243</v>
+      </c>
+      <c r="C39" t="s">
+        <v>366</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39"/>
+      <c r="F39"/>
+      <c r="G39"/>
+      <c r="H39"/>
+      <c r="I39"/>
+      <c r="J39"/>
+      <c r="K39"/>
+      <c r="L39"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>340</v>
+      </c>
+      <c r="B40" t="s">
+        <v>20</v>
+      </c>
+      <c r="C40" t="s">
+        <v>366</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40"/>
+      <c r="F40"/>
+      <c r="G40"/>
+      <c r="H40"/>
+      <c r="I40"/>
+      <c r="J40"/>
+      <c r="K40"/>
+      <c r="L40"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>340</v>
+      </c>
+      <c r="B41" t="s">
+        <v>24</v>
+      </c>
+      <c r="C41" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D41" t="n">
+        <v>140</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.0254716725051756</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.0412174001323173</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.537637452814577</v>
+      </c>
+      <c r="H41"/>
+      <c r="I41"/>
+      <c r="J41"/>
+      <c r="K41" t="n">
+        <v>-0.0553144317541664</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0.106257776764518</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>340</v>
+      </c>
+      <c r="B42" t="s">
+        <v>24</v>
+      </c>
+      <c r="C42" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D42" t="n">
+        <v>81</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.000191123707001848</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.055010236591423</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.997237100004318</v>
+      </c>
+      <c r="H42"/>
+      <c r="I42"/>
+      <c r="J42"/>
+      <c r="K42" t="n">
+        <v>-0.107628940012187</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.108011187426191</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>340</v>
+      </c>
+      <c r="B43" t="s">
+        <v>24</v>
+      </c>
+      <c r="C43" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D43" t="n">
+        <v>131</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.00256460781171256</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.0422138727381663</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.951654159778687</v>
+      </c>
+      <c r="H43"/>
+      <c r="I43"/>
+      <c r="J43"/>
+      <c r="K43" t="n">
+        <v>-0.0801745827550933</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.0853037983785184</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>340</v>
+      </c>
+      <c r="B44" t="s">
+        <v>40</v>
+      </c>
+      <c r="C44" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D44" t="n">
+        <v>55</v>
+      </c>
+      <c r="E44" t="n">
+        <v>-0.1415664030555</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.0757433144775453</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.0673547947121075</v>
+      </c>
+      <c r="H44"/>
+      <c r="I44"/>
+      <c r="J44"/>
+      <c r="K44" t="n">
+        <v>-0.290023299431489</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0.00689049332048836</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>340</v>
+      </c>
+      <c r="B45" t="s">
+        <v>40</v>
+      </c>
+      <c r="C45" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D45" t="n">
+        <v>32</v>
+      </c>
+      <c r="E45" t="n">
+        <v>-0.223926364626869</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.0838682382344966</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.0124187705150574</v>
+      </c>
+      <c r="H45"/>
+      <c r="I45"/>
+      <c r="J45"/>
+      <c r="K45" t="n">
+        <v>-0.388308111566482</v>
+      </c>
+      <c r="L45" t="n">
+        <v>-0.0595446176872553</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>340</v>
+      </c>
+      <c r="B46" t="s">
+        <v>40</v>
+      </c>
+      <c r="C46" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D46" t="n">
+        <v>51</v>
+      </c>
+      <c r="E46" t="n">
+        <v>-0.188270793480401</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.0757885235988591</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.016609188403439</v>
+      </c>
+      <c r="H46"/>
+      <c r="I46"/>
+      <c r="J46"/>
+      <c r="K46" t="n">
+        <v>-0.336816299734165</v>
+      </c>
+      <c r="L46" t="n">
+        <v>-0.0397252872266375</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>340</v>
+      </c>
+      <c r="B47" t="s">
+        <v>54</v>
+      </c>
+      <c r="C47" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D47" t="n">
+        <v>344</v>
+      </c>
+      <c r="E47" t="n">
+        <v>-0.0161886791954185</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.0284059286277115</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.569121074505925</v>
+      </c>
+      <c r="H47"/>
+      <c r="I47"/>
+      <c r="J47"/>
+      <c r="K47" t="n">
+        <v>-0.071864299305733</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0.039486940914896</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>340</v>
+      </c>
+      <c r="B48" t="s">
+        <v>54</v>
+      </c>
+      <c r="C48" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D48" t="n">
+        <v>253</v>
+      </c>
+      <c r="E48" t="n">
+        <v>-0.00833222499215648</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.0328824043913617</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.800174246923656</v>
+      </c>
+      <c r="H48"/>
+      <c r="I48"/>
+      <c r="J48"/>
+      <c r="K48" t="n">
+        <v>-0.0727817375992253</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0.0561172876149124</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>340</v>
+      </c>
+      <c r="B49" t="s">
+        <v>54</v>
+      </c>
+      <c r="C49" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D49" t="n">
+        <v>306</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.000166102230528311</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.0303008036817769</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.995629856151925</v>
+      </c>
+      <c r="H49"/>
+      <c r="I49"/>
+      <c r="J49"/>
+      <c r="K49" t="n">
+        <v>-0.0592234729857543</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0.0595556774468109</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>340</v>
+      </c>
+      <c r="B50" t="s">
+        <v>67</v>
+      </c>
+      <c r="C50" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D50" t="n">
+        <v>136</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.0523161041578691</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.0514497874004185</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.311104018415296</v>
+      </c>
+      <c r="H50"/>
+      <c r="I50"/>
+      <c r="J50"/>
+      <c r="K50" t="n">
+        <v>-0.0485254791469512</v>
+      </c>
+      <c r="L50" t="n">
+        <v>0.153157687462689</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>340</v>
+      </c>
+      <c r="B51" t="s">
+        <v>67</v>
+      </c>
+      <c r="C51" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D51" t="n">
+        <v>92</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.120766452951484</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.0625502567402343</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.0567533169086693</v>
+      </c>
+      <c r="H51"/>
+      <c r="I51"/>
+      <c r="J51"/>
+      <c r="K51" t="n">
+        <v>-0.0018320502593747</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0.243364956162344</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>340</v>
+      </c>
+      <c r="B52" t="s">
+        <v>67</v>
+      </c>
+      <c r="C52" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D52" t="n">
+        <v>128</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.0441917266093737</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.0524150046908572</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.400811701517185</v>
+      </c>
+      <c r="H52"/>
+      <c r="I52"/>
+      <c r="J52"/>
+      <c r="K52" t="n">
+        <v>-0.0585416825847064</v>
+      </c>
+      <c r="L52" t="n">
+        <v>0.146925135803454</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>340</v>
+      </c>
+      <c r="B53" t="s">
+        <v>103</v>
+      </c>
+      <c r="C53" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D53" t="n">
+        <v>675</v>
+      </c>
+      <c r="E53" t="n">
+        <v>-0.00409962275939631</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.0207918883261531</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.84375149890792</v>
+      </c>
+      <c r="H53"/>
+      <c r="I53"/>
+      <c r="J53"/>
+      <c r="K53" t="n">
+        <v>-0.0448517238786565</v>
+      </c>
+      <c r="L53" t="n">
+        <v>0.0366524783598639</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>340</v>
+      </c>
+      <c r="B54" t="s">
+        <v>103</v>
+      </c>
+      <c r="C54" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D54" t="n">
+        <v>458</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.000589714547561613</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.0250429852465854</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.981223556104258</v>
+      </c>
+      <c r="H54"/>
+      <c r="I54"/>
+      <c r="J54"/>
+      <c r="K54" t="n">
+        <v>-0.0484945365357457</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0.049673965630869</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>340</v>
+      </c>
+      <c r="B55" t="s">
+        <v>103</v>
+      </c>
+      <c r="C55" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D55" t="n">
+        <v>616</v>
+      </c>
+      <c r="E55" t="n">
+        <v>-0.0080248800618011</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.0216777552346048</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.711370720555856</v>
+      </c>
+      <c r="H55"/>
+      <c r="I55"/>
+      <c r="J55"/>
+      <c r="K55" t="n">
+        <v>-0.0505132803216265</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0.0344635201980243</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>352</v>
+      </c>
+      <c r="B56" t="s">
+        <v>3241</v>
+      </c>
+      <c r="C56" t="s">
+        <v>366</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56"/>
+      <c r="F56"/>
+      <c r="G56"/>
+      <c r="H56"/>
+      <c r="I56"/>
+      <c r="J56"/>
+      <c r="K56"/>
+      <c r="L56"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>352</v>
+      </c>
+      <c r="B57" t="s">
+        <v>3243</v>
+      </c>
+      <c r="C57" t="s">
+        <v>366</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57"/>
+      <c r="F57"/>
+      <c r="G57"/>
+      <c r="H57"/>
+      <c r="I57"/>
+      <c r="J57"/>
+      <c r="K57"/>
+      <c r="L57"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>352</v>
+      </c>
+      <c r="B58" t="s">
+        <v>20</v>
+      </c>
+      <c r="C58" t="s">
+        <v>366</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58"/>
+      <c r="F58"/>
+      <c r="G58"/>
+      <c r="H58"/>
+      <c r="I58"/>
+      <c r="J58"/>
+      <c r="K58"/>
+      <c r="L58"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>352</v>
+      </c>
+      <c r="B59" t="s">
+        <v>24</v>
+      </c>
+      <c r="C59" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D59" t="n">
+        <v>142</v>
+      </c>
+      <c r="E59" t="n">
+        <v>-0.0163692522466111</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.0451462436586527</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0.717484992839257</v>
+      </c>
+      <c r="H59"/>
+      <c r="I59"/>
+      <c r="J59"/>
+      <c r="K59" t="n">
+        <v>-0.10485588981757</v>
+      </c>
+      <c r="L59" t="n">
+        <v>0.0721173853243483</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>352</v>
+      </c>
+      <c r="B60" t="s">
+        <v>24</v>
+      </c>
+      <c r="C60" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D60" t="n">
+        <v>82</v>
+      </c>
+      <c r="E60" t="n">
+        <v>-0.0221691965853269</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.0579042739740759</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0.702911746581395</v>
+      </c>
+      <c r="H60"/>
+      <c r="I60"/>
+      <c r="J60"/>
+      <c r="K60" t="n">
+        <v>-0.135661573574516</v>
+      </c>
+      <c r="L60" t="n">
+        <v>0.0913231804038618</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>352</v>
+      </c>
+      <c r="B61" t="s">
+        <v>24</v>
+      </c>
+      <c r="C61" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D61" t="n">
+        <v>133</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.00030050278709655</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.0477414431359687</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0.994987906935465</v>
+      </c>
+      <c r="H61"/>
+      <c r="I61"/>
+      <c r="J61"/>
+      <c r="K61" t="n">
+        <v>-0.0932727257594021</v>
+      </c>
+      <c r="L61" t="n">
+        <v>0.0938737313335952</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>352</v>
+      </c>
+      <c r="B62" t="s">
+        <v>40</v>
+      </c>
+      <c r="C62" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D62" t="n">
+        <v>55</v>
+      </c>
+      <c r="E62" t="n">
+        <v>-0.0388152830540266</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.100129632386142</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0.699893125633028</v>
+      </c>
+      <c r="H62"/>
+      <c r="I62"/>
+      <c r="J62"/>
+      <c r="K62" t="n">
+        <v>-0.235069362530864</v>
+      </c>
+      <c r="L62" t="n">
+        <v>0.157438796422811</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>352</v>
+      </c>
+      <c r="B63" t="s">
+        <v>40</v>
+      </c>
+      <c r="C63" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D63" t="n">
+        <v>32</v>
+      </c>
+      <c r="E63" t="n">
+        <v>-0.0568609368357968</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.129830528701411</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0.664665214401096</v>
+      </c>
+      <c r="H63"/>
+      <c r="I63"/>
+      <c r="J63"/>
+      <c r="K63" t="n">
+        <v>-0.311328773090562</v>
+      </c>
+      <c r="L63" t="n">
+        <v>0.197606899418968</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>352</v>
+      </c>
+      <c r="B64" t="s">
+        <v>40</v>
+      </c>
+      <c r="C64" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D64" t="n">
+        <v>51</v>
+      </c>
+      <c r="E64" t="n">
+        <v>-0.0669118021923181</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.107438301540728</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0.536493823557169</v>
+      </c>
+      <c r="H64"/>
+      <c r="I64"/>
+      <c r="J64"/>
+      <c r="K64" t="n">
+        <v>-0.277490873212146</v>
+      </c>
+      <c r="L64" t="n">
+        <v>0.14366726882751</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>352</v>
+      </c>
+      <c r="B65" t="s">
+        <v>54</v>
+      </c>
+      <c r="C65" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D65" t="n">
+        <v>350</v>
+      </c>
+      <c r="E65" t="n">
+        <v>-0.0074012480870389</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.0326004473940253</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0.820536651605983</v>
+      </c>
+      <c r="H65"/>
+      <c r="I65"/>
+      <c r="J65"/>
+      <c r="K65" t="n">
+        <v>-0.0712981249793285</v>
+      </c>
+      <c r="L65" t="n">
+        <v>0.0564956288052507</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>352</v>
+      </c>
+      <c r="B66" t="s">
+        <v>54</v>
+      </c>
+      <c r="C66" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D66" t="n">
+        <v>255</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.00973315378085288</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.0370881353344702</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0.793205672911956</v>
+      </c>
+      <c r="H66"/>
+      <c r="I66"/>
+      <c r="J66"/>
+      <c r="K66" t="n">
+        <v>-0.0629595914747086</v>
+      </c>
+      <c r="L66" t="n">
+        <v>0.0824258990364144</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>352</v>
+      </c>
+      <c r="B67" t="s">
+        <v>54</v>
+      </c>
+      <c r="C67" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D67" t="n">
+        <v>311</v>
+      </c>
+      <c r="E67" t="n">
+        <v>-0.00388238903823931</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.0353640472097041</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0.912653795766756</v>
+      </c>
+      <c r="H67"/>
+      <c r="I67"/>
+      <c r="J67"/>
+      <c r="K67" t="n">
+        <v>-0.0731959215692594</v>
+      </c>
+      <c r="L67" t="n">
+        <v>0.0654311434927808</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>352</v>
+      </c>
+      <c r="B68" t="s">
+        <v>67</v>
+      </c>
+      <c r="C68" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D68" t="n">
+        <v>136</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0.0227403021631089</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.0757450401319123</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0.764481017509522</v>
+      </c>
+      <c r="H68"/>
+      <c r="I68"/>
+      <c r="J68"/>
+      <c r="K68" t="n">
+        <v>-0.125719976495439</v>
+      </c>
+      <c r="L68" t="n">
+        <v>0.171200580821657</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>352</v>
+      </c>
+      <c r="B69" t="s">
+        <v>67</v>
+      </c>
+      <c r="C69" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D69" t="n">
+        <v>92</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0.0110868152096264</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.0731570537493623</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0.879890683161944</v>
+      </c>
+      <c r="H69"/>
+      <c r="I69"/>
+      <c r="J69"/>
+      <c r="K69" t="n">
+        <v>-0.132301010139124</v>
+      </c>
+      <c r="L69" t="n">
+        <v>0.154474640558377</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>352</v>
+      </c>
+      <c r="B70" t="s">
+        <v>67</v>
+      </c>
+      <c r="C70" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D70" t="n">
+        <v>128</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0.0101744128126387</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.0800314331852242</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0.89904522554826</v>
+      </c>
+      <c r="H70"/>
+      <c r="I70"/>
+      <c r="J70"/>
+      <c r="K70" t="n">
+        <v>-0.146687196230401</v>
+      </c>
+      <c r="L70" t="n">
+        <v>0.167036021855678</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>352</v>
+      </c>
+      <c r="B71" t="s">
+        <v>103</v>
+      </c>
+      <c r="C71" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D71" t="n">
+        <v>683</v>
+      </c>
+      <c r="E71" t="n">
+        <v>-0.00613766848228212</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.0257012359280895</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0.811327039440443</v>
+      </c>
+      <c r="H71"/>
+      <c r="I71"/>
+      <c r="J71"/>
+      <c r="K71" t="n">
+        <v>-0.0565120909013376</v>
+      </c>
+      <c r="L71" t="n">
+        <v>0.0442367539367733</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>352</v>
+      </c>
+      <c r="B72" t="s">
+        <v>103</v>
+      </c>
+      <c r="C72" t="s">
+        <v>3245</v>
+      </c>
+      <c r="D72" t="n">
+        <v>461</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0.00108265062444197</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.0288324360067722</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0.970063332452963</v>
+      </c>
+      <c r="H72"/>
+      <c r="I72"/>
+      <c r="J72"/>
+      <c r="K72" t="n">
+        <v>-0.0554289239488316</v>
+      </c>
+      <c r="L72" t="n">
+        <v>0.0575942251977155</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>352</v>
+      </c>
+      <c r="B73" t="s">
+        <v>103</v>
+      </c>
+      <c r="C73" t="s">
+        <v>3246</v>
+      </c>
+      <c r="D73" t="n">
+        <v>623</v>
+      </c>
+      <c r="E73" t="n">
+        <v>-0.00794767296526183</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0.0275678061869019</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0.773218322581104</v>
+      </c>
+      <c r="H73"/>
+      <c r="I73"/>
+      <c r="J73"/>
+      <c r="K73" t="n">
+        <v>-0.0619805730915895</v>
+      </c>
+      <c r="L73" t="n">
+        <v>0.0460852271610659</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>

</xml_diff>